<commit_message>
Add scripts for generating salary figures and LaTeX tables for descriptive statistics and inferential results
- Created a Python script `export_figures.py` to generate histograms and boxplots for average salaries in PB and RN, saving them as PDF and SVG files.
- Added LaTeX table `tab_descritiva_salario.tex` for descriptive statistics of average formal salary samples.
- Introduced LaTeX table `tab_inferencia.tex` summarizing inferential results with statistical tests and decisions.
</commit_message>
<xml_diff>
--- a/data/Estatisticas_Descritivas.xlsx
+++ b/data/Estatisticas_Descritivas.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,54 +420,54 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Mediana</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>variância</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Desvio Padrão</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Mínimo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Máximo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>IDEB – Anos iniciais do ensino fundamental (Rede pública)</t>
         </is>
@@ -513,7 +501,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Percentual da população com rendimento nominal mensal per capita de até 1/2 salário mínimo</t>
         </is>
@@ -547,7 +535,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Salário médio mensal dos trabalhadores formais</t>
         </is>
@@ -595,54 +583,54 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Mediana</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>variância</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Desvio Padrão</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Mínimo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Máximo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>IDEB – Anos iniciais do ensino fundamental (Rede pública)</t>
         </is>
@@ -676,7 +664,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Percentual da população com rendimento nominal mensal per capita de até 1/2 salário mínimo</t>
         </is>
@@ -710,7 +698,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Salário médio mensal dos trabalhadores formais</t>
         </is>
@@ -758,54 +746,54 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Mediana</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>variância</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Desvio Padrão</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Mínimo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Máximo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>IDEB – Anos iniciais do ensino fundamental (Rede pública)</t>
         </is>
@@ -839,7 +827,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Percentual da população com rendimento nominal mensal per capita de até 1/2 salário mínimo (%)</t>
         </is>
@@ -873,7 +861,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Salário médio mensal dos trabalhadores formais</t>
         </is>
@@ -921,54 +909,54 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Mediana</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>variância</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Desvio Padrão</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Mínimo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Máximo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>IDEB – Anos iniciais do ensino fundamental (Rede pública)</t>
         </is>
@@ -1002,7 +990,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Percentual da população com rendimento nominal mensal per capita de até 1/2 salário mínimo (%)</t>
         </is>
@@ -1036,7 +1024,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Salário médio mensal dos trabalhadores formais</t>
         </is>

</xml_diff>